<commit_message>
[modify] finish game flow.
</commit_message>
<xml_diff>
--- a/DemoDesign/Config/monster.xlsx
+++ b/DemoDesign/Config/monster.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29127"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A6BB49D1-1EEA-4425-AB06-C8870249A7E3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2B98D674-F547-4AFE-8F6D-A47F8CAD9F40}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="46" uniqueCount="45">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="46" uniqueCount="35">
   <si>
     <t>int</t>
   </si>
@@ -130,37 +130,6 @@
   <si>
     <t>20</t>
     <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>30</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>40</t>
-  </si>
-  <si>
-    <t>50</t>
-  </si>
-  <si>
-    <t>60</t>
-  </si>
-  <si>
-    <t>70</t>
-  </si>
-  <si>
-    <t>80</t>
-  </si>
-  <si>
-    <t>90</t>
-  </si>
-  <si>
-    <t>100</t>
-  </si>
-  <si>
-    <t>110</t>
-  </si>
-  <si>
-    <t>120</t>
   </si>
   <si>
     <t>M01</t>
@@ -668,7 +637,7 @@
         <v>2</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>44</v>
+        <v>34</v>
       </c>
     </row>
     <row r="3" spans="1:3" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
@@ -684,10 +653,10 @@
     </row>
     <row r="4" spans="1:3" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="2" t="s">
-        <v>33</v>
+        <v>23</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>22</v>
+        <v>12</v>
       </c>
       <c r="C4" s="2" t="s">
         <v>11</v>
@@ -695,112 +664,112 @@
     </row>
     <row r="5" spans="1:3" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="2" t="s">
-        <v>34</v>
+        <v>24</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>23</v>
+        <v>13</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
     </row>
     <row r="6" spans="1:3" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="2" t="s">
-        <v>35</v>
+        <v>25</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>24</v>
+        <v>14</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
     </row>
     <row r="7" spans="1:3" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="2" t="s">
-        <v>36</v>
+        <v>26</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>25</v>
+        <v>15</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
     </row>
     <row r="8" spans="1:3" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="2" t="s">
-        <v>37</v>
+        <v>27</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>26</v>
+        <v>16</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>15</v>
+        <v>11</v>
       </c>
     </row>
     <row r="9" spans="1:3" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="2" t="s">
-        <v>38</v>
+        <v>28</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>27</v>
+        <v>17</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>16</v>
+        <v>11</v>
       </c>
     </row>
     <row r="10" spans="1:3" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="2" t="s">
-        <v>39</v>
+        <v>29</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>28</v>
+        <v>18</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>17</v>
+        <v>11</v>
       </c>
     </row>
     <row r="11" spans="1:3" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="2" t="s">
-        <v>40</v>
+        <v>30</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>29</v>
+        <v>19</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>18</v>
+        <v>11</v>
       </c>
     </row>
     <row r="12" spans="1:3" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="2" t="s">
-        <v>41</v>
+        <v>31</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>19</v>
+        <v>11</v>
       </c>
     </row>
     <row r="13" spans="1:3" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" s="2" t="s">
-        <v>42</v>
+        <v>32</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>31</v>
+        <v>21</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>20</v>
+        <v>11</v>
       </c>
     </row>
     <row r="14" spans="1:3" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14" s="2" t="s">
-        <v>43</v>
+        <v>33</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>32</v>
+        <v>22</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>21</v>
+        <v>11</v>
       </c>
     </row>
   </sheetData>

</xml_diff>